<commit_message>
Fix AKBANK KS: decimal parsing - use dot as decimal separator not thousands
The numbers after KS: use dots as decimal separators, not thousands separators.
Fixed parsing to preserve dots as decimals: 51,516.94 TL total (not 4.7M)

01-10.07: 16,414.39 TL
11-20.07: 17,035.74 TL
21-31.07: 18,066.81 TL

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013XirDLHEgVkT9Fvb27rTq6
</commit_message>
<xml_diff>
--- a/AKBANK-KS_Satirlari-Temmuz2026.xlsx
+++ b/AKBANK-KS_Satirlari-Temmuz2026.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>4792927</v>
+        <v>51516.93999999999</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>113266</v>
+        <v>1433.26</v>
       </c>
     </row>
     <row r="6">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>148476</v>
+        <v>1549.92</v>
       </c>
     </row>
     <row r="7">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>141006</v>
+        <v>1807.05</v>
       </c>
     </row>
     <row r="8">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>149468</v>
+        <v>1808.51</v>
       </c>
     </row>
     <row r="9">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>186831</v>
+        <v>1868.31</v>
       </c>
     </row>
     <row r="10">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>148167</v>
+        <v>1574.64</v>
       </c>
     </row>
     <row r="11">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>158550</v>
+        <v>1585.5</v>
       </c>
     </row>
     <row r="12">
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>115050</v>
+        <v>1448.94</v>
       </c>
     </row>
     <row r="13">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>138634</v>
+        <v>1498.93</v>
       </c>
     </row>
     <row r="14">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>183933</v>
+        <v>1839.33</v>
       </c>
     </row>
     <row r="15">
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>1483381</v>
+        <v>16414.39</v>
       </c>
     </row>
     <row r="17">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>174694</v>
+        <v>1790.77</v>
       </c>
     </row>
     <row r="19">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>175253</v>
+        <v>1877.72</v>
       </c>
     </row>
     <row r="20">
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>166819</v>
+        <v>1919.83</v>
       </c>
     </row>
     <row r="21">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>143089</v>
+        <v>1466.44</v>
       </c>
     </row>
     <row r="22">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>168285</v>
+        <v>1706.88</v>
       </c>
     </row>
     <row r="23">
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>171874</v>
+        <v>1758.79</v>
       </c>
     </row>
     <row r="24">
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>144917</v>
+        <v>1736.18</v>
       </c>
     </row>
     <row r="25">
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>151600</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="26">
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>146677</v>
+        <v>1466.77</v>
       </c>
     </row>
     <row r="27">
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>179636</v>
+        <v>1796.36</v>
       </c>
     </row>
     <row r="28">
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>1622844</v>
+        <v>17035.74</v>
       </c>
     </row>
     <row r="30">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>171653</v>
+        <v>1762.79</v>
       </c>
     </row>
     <row r="32">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>139432</v>
+        <v>1394.32</v>
       </c>
     </row>
     <row r="33">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>122657</v>
+        <v>1409.63</v>
       </c>
     </row>
     <row r="34">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>164839</v>
+        <v>1840.27</v>
       </c>
     </row>
     <row r="35">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>171390</v>
+        <v>1734.96</v>
       </c>
     </row>
     <row r="36">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>163385</v>
+        <v>1698.11</v>
       </c>
     </row>
     <row r="37">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>145924</v>
+        <v>1888.99</v>
       </c>
     </row>
     <row r="38">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>163575</v>
+        <v>1635.75</v>
       </c>
     </row>
     <row r="39">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>171727</v>
+        <v>1717.27</v>
       </c>
     </row>
     <row r="40">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>128392</v>
+        <v>1283.92</v>
       </c>
     </row>
     <row r="41">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B41" s="6" t="n">
-        <v>143728</v>
+        <v>1700.8</v>
       </c>
     </row>
     <row r="42">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>1686702</v>
+        <v>18066.81</v>
       </c>
     </row>
     <row r="44">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="B44" s="10" t="n">
-        <v>4792927</v>
+        <v>51516.93999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>